<commit_message>
Add city markers and full-size photo viewer from the updated reference
The owner's updated example adds blue city markers (Gurgaon, Manesar) with
a City legend entry, and a lightbox for card photos. Made generic:

- reference/billboard-plan-example.html replaced with the updated file
- template: cities (markers, legend, Show all sites bounds) and the photo
  lightbox (arrows, Escape, backdrop click, focus returns to the card)
- core: plan.cities in the schema, resolver and planToFile; spreadsheet
  Plan sheet City rows ("Manesar: 28.3540, 76.9395")
- app: Cities section under Plan details; sites template gains a City row
- example plan.yaml and fixture list Gurgaon and Manesar
- tests: reference data CITIES match; e2e city markers, lightbox, and a
  text comparison of the built page against the reference

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/sites-template.xlsx
+++ b/templates/sites-template.xlsx
@@ -479,7 +479,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C18"/>
+  <dimension ref="A1:C19"/>
   <cols>
     <col min="1" max="1" width="18.83203125" customWidth="1"/>
     <col min="2" max="2" width="30.83203125" customWidth="1"/>
@@ -664,13 +664,13 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Note</v>
+        <v>City</v>
       </c>
       <c r="B17" t="str">
         <v/>
       </c>
       <c r="C17" t="str">
-        <v>A line under the table. Add more Note rows for more lines</v>
+        <v>A blue city marker with its name, written as Name: coordinates, e.g. Manesar: 28.3540, 76.9395. Add more City rows for more cities</v>
       </c>
     </row>
     <row r="18">
@@ -681,12 +681,23 @@
         <v/>
       </c>
       <c r="C18" t="str">
+        <v>A line under the table. Add more Note rows for more lines</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>Note</v>
+      </c>
+      <c r="B19" t="str">
+        <v/>
+      </c>
+      <c r="C19" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C18"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C19"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>